<commit_message>
Integrar Universo Ramos y conservar historial de muestras
</commit_message>
<xml_diff>
--- a/Sheet1.xlsx
+++ b/Sheet1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miguel.arroyo\Desktop\macros\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miguel.arroyo\Desktop\Proyectos\macros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B81E94B-EA34-46C6-B391-FC0C0F01281A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9971BFD4-60C1-4E64-8FAB-4ED47156C1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,9 +17,6 @@
     <sheet name="Hoja1" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId4"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1916" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1883" uniqueCount="378">
   <si>
     <t>ID Cliente</t>
   </si>
@@ -1167,6 +1164,9 @@
   </si>
   <si>
     <t>S37</t>
+  </si>
+  <si>
+    <t>82-102088-17</t>
   </si>
 </sst>
 </file>
@@ -1711,7 +1711,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1756,6 +1756,13 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1812,22 +1819,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Hoja1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2094,14 +2085,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125"/>
+    <col min="6" max="6" width="11.42578125" style="18"/>
     <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2121,7 +2112,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="16" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -2136,444 +2127,257 @@
       <c r="B2" s="14" t="s">
         <v>376</v>
       </c>
-      <c r="C2" s="1" t="str">
+      <c r="C2" s="1" t="e">
         <f>VLOOKUP(E2,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
+        <v>#N/A</v>
       </c>
       <c r="D2" s="2">
-        <f ca="1">TODAY()</f>
-        <v>46272</v>
+        <f t="shared" ref="D2:D12" ca="1" si="0">TODAY()</f>
+        <v>46315</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="F2" s="2">
-        <v>700</v>
+        <v>377</v>
+      </c>
+      <c r="F2" s="16">
+        <v>300</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <f>IFERROR(VLOOKUP(C3,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C3" s="1" t="str">
-        <f>VLOOKUP(E3,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D3" s="2">
-        <f t="shared" ref="D3:D13" ca="1" si="0">TODAY()</f>
-        <v>46272</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F3" s="2">
-        <v>300</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="2"/>
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <f>IFERROR(VLOOKUP(C4,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C4" s="1" t="str">
-        <f>VLOOKUP(E4,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D4" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F4" s="2">
-        <v>900</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <f>IFERROR(VLOOKUP(C5,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C5" s="1" t="str">
-        <f>VLOOKUP(E5,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D5" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F5" s="2">
-        <v>1050</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <f>IFERROR(VLOOKUP(C6,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C6" s="1" t="str">
-        <f>VLOOKUP(E6,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D6" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="F6" s="2">
-        <v>800</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <f>IFERROR(VLOOKUP(C7,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C7" s="1" t="str">
-        <f>VLOOKUP(E7,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D7" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F7" s="2">
-        <v>800</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <f>IFERROR(VLOOKUP(C8,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C8" s="1" t="str">
-        <f>VLOOKUP(E8,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D8" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F8" s="2">
-        <v>1600</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <f>IFERROR(VLOOKUP(C9,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C9" s="1" t="str">
-        <f>VLOOKUP(E9,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D9" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="2">
-        <v>400</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <f>IFERROR(VLOOKUP(C10,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C10" s="1" t="str">
-        <f>VLOOKUP(E10,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D10" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F10" s="2">
-        <v>1000</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <f>IFERROR(VLOOKUP(C11,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C11" s="1" t="str">
-        <f>VLOOKUP(E11,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D11" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F11" s="2">
-        <v>1200</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>375</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <f>IFERROR(VLOOKUP(C12,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C12" s="1" t="str">
-        <f>VLOOKUP(E12,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D12" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="F12" s="2">
-        <v>300</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <f>IFERROR(VLOOKUP(C13,#REF!,2,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="C13" s="1" t="str">
-        <f>VLOOKUP(E13,Hoja1!D:L,9,0)</f>
-        <v>DAIKIN USA</v>
-      </c>
-      <c r="D13" s="2">
-        <f t="shared" ca="1" si="0"/>
-        <v>46272</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="F13" s="2">
-        <v>300</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="24" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="14"/>
       <c r="C14" s="1"/>
       <c r="D14" s="2"/>
       <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="F14" s="17"/>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="1:9" ht="24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="14"/>
       <c r="C15" s="1"/>
       <c r="D15" s="2"/>
       <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
+      <c r="F15" s="17"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="1:9" ht="24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="14"/>
       <c r="C16" s="1"/>
       <c r="D16" s="2"/>
       <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
+      <c r="F16" s="17"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="14"/>
       <c r="C17" s="1"/>
       <c r="D17" s="2"/>
       <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
+      <c r="F17" s="17"/>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="14"/>
       <c r="C18" s="1"/>
       <c r="D18" s="2"/>
       <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
+      <c r="F18" s="17"/>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="14"/>
       <c r="C19" s="1"/>
       <c r="D19" s="2"/>
       <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
+      <c r="F19" s="17"/>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="14"/>
       <c r="C20" s="1"/>
       <c r="D20" s="2"/>
       <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
+      <c r="F20" s="17"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="14"/>
       <c r="C21" s="1"/>
       <c r="D21" s="2"/>
       <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+      <c r="F21" s="17"/>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="14"/>
       <c r="C22" s="1"/>
       <c r="D22" s="2"/>
       <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
+      <c r="F22" s="17"/>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="14"/>
       <c r="C23" s="1"/>
       <c r="D23" s="2"/>
       <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
+      <c r="F23" s="17"/>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="14"/>
       <c r="C24" s="1"/>
       <c r="D24" s="2"/>
       <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
+      <c r="F24" s="17"/>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="14"/>
       <c r="C25" s="1"/>
       <c r="D25" s="2"/>
       <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
+      <c r="F25" s="17"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="14"/>
       <c r="C26" s="1"/>
       <c r="D26" s="2"/>
       <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
+      <c r="F26" s="17"/>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="14"/>
       <c r="C27" s="1"/>
       <c r="D27" s="2"/>
       <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
+      <c r="F27" s="17"/>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="14"/>
       <c r="C28" s="1"/>
       <c r="D28" s="2"/>
       <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
+      <c r="F28" s="17"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2582,7 +2386,7 @@
       <c r="C29" s="1"/>
       <c r="D29" s="2"/>
       <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
+      <c r="F29" s="17"/>
       <c r="G29" s="1"/>
     </row>
     <row r="30" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2591,7 +2395,7 @@
       <c r="C30" s="1"/>
       <c r="D30" s="2"/>
       <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
+      <c r="F30" s="17"/>
       <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2600,7 +2404,7 @@
       <c r="C31" s="1"/>
       <c r="D31" s="2"/>
       <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
+      <c r="F31" s="17"/>
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2609,7 +2413,7 @@
       <c r="C32" s="1"/>
       <c r="D32" s="2"/>
       <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
+      <c r="F32" s="17"/>
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2618,7 +2422,7 @@
       <c r="C33" s="1"/>
       <c r="D33" s="2"/>
       <c r="E33" s="15"/>
-      <c r="F33" s="15"/>
+      <c r="F33" s="17"/>
       <c r="G33" s="1"/>
     </row>
     <row r="34" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2627,7 +2431,7 @@
       <c r="C34" s="1"/>
       <c r="D34" s="2"/>
       <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
+      <c r="F34" s="17"/>
       <c r="G34" s="1"/>
     </row>
     <row r="35" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2636,7 +2440,7 @@
       <c r="C35" s="1"/>
       <c r="D35" s="2"/>
       <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
+      <c r="F35" s="17"/>
       <c r="G35" s="1"/>
     </row>
     <row r="36" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2645,7 +2449,7 @@
       <c r="C36" s="1"/>
       <c r="D36" s="2"/>
       <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
+      <c r="F36" s="17"/>
       <c r="G36" s="1"/>
     </row>
     <row r="37" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2654,7 +2458,7 @@
       <c r="C37" s="1"/>
       <c r="D37" s="2"/>
       <c r="E37" s="15"/>
-      <c r="F37" s="15"/>
+      <c r="F37" s="17"/>
       <c r="G37" s="1"/>
     </row>
     <row r="38" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2663,7 +2467,7 @@
       <c r="C38" s="1"/>
       <c r="D38" s="2"/>
       <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
+      <c r="F38" s="17"/>
       <c r="G38" s="1"/>
     </row>
     <row r="39" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2672,7 +2476,7 @@
       <c r="C39" s="1"/>
       <c r="D39" s="2"/>
       <c r="E39" s="15"/>
-      <c r="F39" s="15"/>
+      <c r="F39" s="17"/>
       <c r="G39" s="1"/>
     </row>
     <row r="40" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2681,7 +2485,7 @@
       <c r="C40" s="1"/>
       <c r="D40" s="2"/>
       <c r="E40" s="15"/>
-      <c r="F40" s="15"/>
+      <c r="F40" s="17"/>
       <c r="G40" s="1"/>
     </row>
     <row r="41" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2690,7 +2494,7 @@
       <c r="C41" s="1"/>
       <c r="D41" s="2"/>
       <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
+      <c r="F41" s="17"/>
       <c r="G41" s="1"/>
     </row>
     <row r="42" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2699,7 +2503,7 @@
       <c r="C42" s="1"/>
       <c r="D42" s="2"/>
       <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
+      <c r="F42" s="17"/>
       <c r="G42" s="1"/>
     </row>
     <row r="43" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2708,7 +2512,7 @@
       <c r="C43" s="1"/>
       <c r="D43" s="2"/>
       <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
+      <c r="F43" s="17"/>
       <c r="G43" s="1"/>
     </row>
     <row r="44" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2717,7 +2521,7 @@
       <c r="C44" s="1"/>
       <c r="D44" s="2"/>
       <c r="E44" s="15"/>
-      <c r="F44" s="15"/>
+      <c r="F44" s="17"/>
       <c r="G44" s="1"/>
     </row>
     <row r="45" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2726,7 +2530,7 @@
       <c r="C45" s="1"/>
       <c r="D45" s="2"/>
       <c r="E45" s="15"/>
-      <c r="F45" s="15"/>
+      <c r="F45" s="17"/>
       <c r="G45" s="1"/>
     </row>
     <row r="46" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2735,7 +2539,7 @@
       <c r="C46" s="1"/>
       <c r="D46" s="2"/>
       <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
+      <c r="F46" s="17"/>
       <c r="G46" s="1"/>
     </row>
     <row r="47" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2744,7 +2548,7 @@
       <c r="C47" s="1"/>
       <c r="D47" s="2"/>
       <c r="E47" s="15"/>
-      <c r="F47" s="15"/>
+      <c r="F47" s="17"/>
       <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2753,7 +2557,7 @@
       <c r="C48" s="1"/>
       <c r="D48" s="2"/>
       <c r="E48" s="15"/>
-      <c r="F48" s="15"/>
+      <c r="F48" s="17"/>
       <c r="G48" s="1"/>
     </row>
     <row r="49" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2762,7 +2566,7 @@
       <c r="C49" s="1"/>
       <c r="D49" s="2"/>
       <c r="E49" s="15"/>
-      <c r="F49" s="15"/>
+      <c r="F49" s="17"/>
       <c r="G49" s="1"/>
     </row>
     <row r="50" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2771,7 +2575,7 @@
       <c r="C50" s="1"/>
       <c r="D50" s="2"/>
       <c r="E50" s="15"/>
-      <c r="F50" s="15"/>
+      <c r="F50" s="17"/>
       <c r="G50" s="1"/>
     </row>
     <row r="51" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2780,7 +2584,7 @@
       <c r="C51" s="1"/>
       <c r="D51" s="2"/>
       <c r="E51" s="15"/>
-      <c r="F51" s="15"/>
+      <c r="F51" s="17"/>
       <c r="G51" s="1"/>
     </row>
     <row r="52" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2789,7 +2593,7 @@
       <c r="C52" s="1"/>
       <c r="D52" s="2"/>
       <c r="E52" s="15"/>
-      <c r="F52" s="15"/>
+      <c r="F52" s="17"/>
       <c r="G52" s="1"/>
     </row>
     <row r="53" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2798,7 +2602,7 @@
       <c r="C53" s="1"/>
       <c r="D53" s="2"/>
       <c r="E53" s="15"/>
-      <c r="F53" s="15"/>
+      <c r="F53" s="17"/>
       <c r="G53" s="1"/>
     </row>
     <row r="54" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2807,7 +2611,7 @@
       <c r="C54" s="1"/>
       <c r="D54" s="2"/>
       <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
+      <c r="F54" s="17"/>
       <c r="G54" s="1"/>
     </row>
     <row r="55" spans="1:7" ht="21" x14ac:dyDescent="0.25">
@@ -2816,21 +2620,13 @@
       <c r="C55" s="1"/>
       <c r="D55" s="2"/>
       <c r="E55" s="15"/>
-      <c r="F55" s="15"/>
+      <c r="F55" s="17"/>
       <c r="G55" s="1"/>
-    </row>
-    <row r="56" spans="1:7" ht="21" x14ac:dyDescent="0.25">
-      <c r="A56" s="1"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>